<commit_message>
backtest score error fixed
</commit_message>
<xml_diff>
--- a/CATI/saved_states/NABIL_future_30_day_forecast.xlsx
+++ b/CATI/saved_states/NABIL_future_30_day_forecast.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,11 +443,6 @@
           <t>Signal</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -458,9 +453,6 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>0.3606313031927393</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -471,9 +463,6 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>0.3606313031927393</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -484,9 +473,6 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>0.3606313031927393</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -497,9 +483,6 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>0.3606313031927393</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -510,9 +493,6 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>0.3606313031927393</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -523,9 +503,6 @@
           <t>SELL</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>0.3606313031927393</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -535,9 +512,6 @@
         <is>
           <t>SELL</t>
         </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.3606312833245244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>